<commit_message>
Add four INDUS item factors and fix the LALKUMBH item name spacing
</commit_message>
<xml_diff>
--- a/source data/Item Master Supplement.xlsx
+++ b/source data/Item Master Supplement.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>LALKUMBH  RD  (5 X  5 KGS NON WOVEN BAG)</t>
+          <t>LALKUMBH  RD  (5 X  5 KGS NON WOVEN BAG)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1075,6 +1075,70 @@
         <v>25</v>
       </c>
       <c r="D41" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>INDUS BLACKCURRENT 25 DC TAG TBGS POUCH</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>25</v>
+      </c>
+      <c r="D42" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>INDUS LEMON 25 DC TAG TBGS POUCH</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>25</v>
+      </c>
+      <c r="D43" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>INDUS MANGO &amp; STRAWBERRY 25 DC TAG TBGS POUCH</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>25</v>
+      </c>
+      <c r="D44" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>INDUS WILD BERRIES 25 DC TAG TBGS POUCH</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>25</v>
+      </c>
+      <c r="D45" t="n">
         <v>25</v>
       </c>
     </row>

</xml_diff>